<commit_message>
finished the reset all data button
no longer requires going into file system to reset the data. created a excel with the proper formatting for the initial 11 campuses
</commit_message>
<xml_diff>
--- a/res/testFile.xlsx
+++ b/res/testFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erfantavassoli/Desktop/CS 1d Project 1/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erfan\Documents\CS1D project 1\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C67125-5A1A-3E45-9E60-693A1C8194BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F942A2-1A65-4679-A12D-B0E72124EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18000" yWindow="820" windowWidth="18020" windowHeight="21360" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
+    <workbookView xWindow="12540" yWindow="7680" windowWidth="28296" windowHeight="14916" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
   </bookViews>
   <sheets>
     <sheet name="souvenirs" sheetId="1" r:id="rId1"/>
@@ -37,40 +37,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>campusID</t>
   </si>
   <si>
-    <t>souvenir name</t>
-  </si>
-  <si>
     <t>price</t>
   </si>
   <si>
-    <t>campus name</t>
-  </si>
-  <si>
-    <t>testing campus</t>
-  </si>
-  <si>
-    <t>testSouvenir1</t>
-  </si>
-  <si>
-    <t>testSouvenir2</t>
+    <t>souvenirName</t>
+  </si>
+  <si>
+    <t>campusName</t>
+  </si>
+  <si>
+    <t>University of Texas</t>
+  </si>
+  <si>
+    <t>Coaster set</t>
+  </si>
+  <si>
+    <t>Face paint</t>
+  </si>
+  <si>
+    <t>Sports chair</t>
+  </si>
+  <si>
+    <t>California State University, Fullerton</t>
+  </si>
+  <si>
+    <t>Canopy</t>
+  </si>
+  <si>
+    <t>Flag</t>
+  </si>
+  <si>
+    <t>Keychain</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,8 +117,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,41 +458,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1B26B2-90DC-AD40-AA73-10DECA69AE20}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C2" s="1">
+        <v>14.94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
-        <v>15</v>
-      </c>
+      <c r="C3" s="1">
+        <v>7.53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1">
+        <v>85.99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1">
+        <v>96.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>15.76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>7.98</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F8" s="2"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F9" s="2"/>
+      <c r="G9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -472,10 +555,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE804BB-079C-DE43-A129-6624CA4948A8}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,12 +566,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed bugs in fileupload
</commit_message>
<xml_diff>
--- a/res/testFile.xlsx
+++ b/res/testFile.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erfan\Documents\CS1D project 1\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F942A2-1A65-4679-A12D-B0E72124EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFED57E5-55FF-42ED-BCC3-1075988BAF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12540" yWindow="7680" windowWidth="28296" windowHeight="14916" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
+    <workbookView xWindow="1668" yWindow="1392" windowWidth="17988" windowHeight="14916" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
   </bookViews>
   <sheets>
-    <sheet name="souvenirs" sheetId="1" r:id="rId1"/>
-    <sheet name="campusList" sheetId="2" r:id="rId2"/>
+    <sheet name="campusList" sheetId="2" r:id="rId1"/>
+    <sheet name="souvenirs" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -120,10 +120,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,6 +457,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE804BB-079C-DE43-A129-6624CA4948A8}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1B26B2-90DC-AD40-AA73-10DECA69AE20}">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -551,38 +585,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE804BB-079C-DE43-A129-6624CA4948A8}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
updated file upload logic to add campusDistances as well
</commit_message>
<xml_diff>
--- a/res/testFile.xlsx
+++ b/res/testFile.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erfan\Documents\CS1D project 1\res\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erfantavassoli/Desktop/CS 1d Project 1/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFED57E5-55FF-42ED-BCC3-1075988BAF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FA6049-30D2-214D-883E-62E89E7F6B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1668" yWindow="1392" windowWidth="17988" windowHeight="14916" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
+    <workbookView xWindow="4020" yWindow="1720" windowWidth="13140" windowHeight="19480" activeTab="2" xr2:uid="{35F733E3-80AA-AD43-BF61-482DE484EDDA}"/>
   </bookViews>
   <sheets>
     <sheet name="campusList" sheetId="2" r:id="rId1"/>
     <sheet name="souvenirs" sheetId="1" r:id="rId2"/>
+    <sheet name="distances" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>campusID</t>
   </si>
@@ -73,6 +74,15 @@
   </si>
   <si>
     <t>Keychain</t>
+  </si>
+  <si>
+    <t>distance</t>
+  </si>
+  <si>
+    <t>campusID2</t>
+  </si>
+  <si>
+    <t>campusID1</t>
   </si>
 </sst>
 </file>
@@ -105,7 +115,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -113,17 +123,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -459,9 +584,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE804BB-079C-DE43-A129-6624CA4948A8}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -469,17 +594,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
@@ -493,9 +618,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1B26B2-90DC-AD40-AA73-10DECA69AE20}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -506,9 +631,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -517,9 +642,9 @@
         <v>14.94</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -528,9 +653,9 @@
         <v>7.53</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -539,9 +664,9 @@
         <v>85.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -550,9 +675,9 @@
         <v>96.75</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -561,9 +686,9 @@
         <v>15.76</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -574,13 +699,353 @@
       <c r="F7" s="2"/>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F8" s="2"/>
       <c r="G8" s="3"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F9" s="2"/>
       <c r="G9" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11CB3235-EEE6-6246-B078-D42930BA17CE}">
+  <dimension ref="A1:K30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="42.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="8">
+        <v>12</v>
+      </c>
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="11">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2</v>
+      </c>
+      <c r="C3" s="12">
+        <v>2968</v>
+      </c>
+      <c r="J3" s="6"/>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="11">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="12">
+        <v>2013</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="11">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="12">
+        <v>2231</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="11">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5">
+        <v>5</v>
+      </c>
+      <c r="C6" s="12">
+        <v>29.3</v>
+      </c>
+      <c r="J6" s="6"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="11">
+        <v>12</v>
+      </c>
+      <c r="B7" s="5">
+        <v>6</v>
+      </c>
+      <c r="C7" s="12">
+        <v>20.2</v>
+      </c>
+      <c r="J7" s="6"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="11">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5">
+        <v>7</v>
+      </c>
+      <c r="C8" s="12">
+        <v>47.9</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="11">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5">
+        <v>8</v>
+      </c>
+      <c r="C9" s="12">
+        <v>2229</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="11">
+        <v>12</v>
+      </c>
+      <c r="B10" s="5">
+        <v>9</v>
+      </c>
+      <c r="C10" s="12">
+        <v>884</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="11">
+        <v>12</v>
+      </c>
+      <c r="B11" s="5">
+        <v>10</v>
+      </c>
+      <c r="C11" s="12">
+        <v>368</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="11">
+        <v>12</v>
+      </c>
+      <c r="B12" s="4">
+        <v>11</v>
+      </c>
+      <c r="C12" s="12">
+        <v>1963</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="11">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4">
+        <v>13</v>
+      </c>
+      <c r="C13" s="12">
+        <v>1758</v>
+      </c>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="11">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+      <c r="C14" s="12">
+        <v>1007</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="11">
+        <v>13</v>
+      </c>
+      <c r="B15" s="5">
+        <v>2</v>
+      </c>
+      <c r="C15" s="12">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="11">
+        <v>13</v>
+      </c>
+      <c r="B16" s="5">
+        <v>3</v>
+      </c>
+      <c r="C16" s="12">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="11">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5">
+        <v>4</v>
+      </c>
+      <c r="C17" s="12">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="11">
+        <v>13</v>
+      </c>
+      <c r="B18" s="5">
+        <v>5</v>
+      </c>
+      <c r="C18" s="12">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="11">
+        <v>13</v>
+      </c>
+      <c r="B19" s="5">
+        <v>6</v>
+      </c>
+      <c r="C19" s="12">
+        <v>1375</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="7"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="11">
+        <v>13</v>
+      </c>
+      <c r="B20" s="5">
+        <v>7</v>
+      </c>
+      <c r="C20" s="12">
+        <v>1396</v>
+      </c>
+      <c r="J20" s="6"/>
+      <c r="K20" s="7"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="11">
+        <v>13</v>
+      </c>
+      <c r="B21" s="5">
+        <v>8</v>
+      </c>
+      <c r="C21" s="12">
+        <v>1368</v>
+      </c>
+      <c r="J21" s="6"/>
+      <c r="K21" s="7"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="11">
+        <v>13</v>
+      </c>
+      <c r="B22" s="5">
+        <v>9</v>
+      </c>
+      <c r="C22" s="12">
+        <v>2073</v>
+      </c>
+      <c r="J22" s="6"/>
+      <c r="K22" s="7"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="11">
+        <v>13</v>
+      </c>
+      <c r="B23" s="4">
+        <v>10</v>
+      </c>
+      <c r="C23" s="12">
+        <v>1720</v>
+      </c>
+      <c r="J23" s="6"/>
+      <c r="K23" s="7"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="13">
+        <v>13</v>
+      </c>
+      <c r="B24" s="14">
+        <v>11</v>
+      </c>
+      <c r="C24" s="15">
+        <v>1183</v>
+      </c>
+      <c r="J24" s="6"/>
+      <c r="K24" s="7"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J25" s="6"/>
+      <c r="K25" s="7"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J26" s="6"/>
+      <c r="K26" s="7"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J27" s="6"/>
+      <c r="K27" s="7"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J28" s="6"/>
+      <c r="K28" s="7"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J29" s="6"/>
+      <c r="K29" s="7"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J30" s="6"/>
+      <c r="K30" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>